<commit_message>
Enhance WinProb UI, analytics, and exports with stakeholder-ready readouts.
Modularize the app into focused packages, add executive summary and glossary navigation, fix Plotly/PDF/export issues, improve runner-up tie-breaks, and escape dynamic HTML so wizard and KPI cards render correctly.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/(incrementality)260311_TTD_LAL.xlsx
+++ b/(incrementality)260311_TTD_LAL.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10621"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://twdc-my.sharepoint.com/personal/shirley_deng_disney_com/Documents/Documents/winning_prob/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="259" documentId="8_{904D1800-88DA-A24D-B962-31B32AD975CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8478904B-1590-4643-98B8-65CEB0A85A7F}"/>
+  <xr:revisionPtr revIDLastSave="292" documentId="8_{904D1800-88DA-A24D-B962-31B32AD975CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{144FB372-E45B-FC40-AFCA-A3E512E585C2}"/>
   <bookViews>
-    <workbookView xWindow="2940" yWindow="3520" windowWidth="25620" windowHeight="19740" xr2:uid="{2B257662-BBB0-7E4F-AE21-5DF4D2EB5C7F}"/>
+    <workbookView xWindow="2940" yWindow="720" windowWidth="25620" windowHeight="19740" xr2:uid="{2B257662-BBB0-7E4F-AE21-5DF4D2EB5C7F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -107,7 +107,7 @@
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="0.000%"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
-    <numFmt numFmtId="169" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="166" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="10" x14ac:knownFonts="1">
     <font>
@@ -118,12 +118,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
@@ -150,30 +144,36 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
       <b/>
       <sz val="12"/>
       <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
     <font>
       <sz val="12"/>
-      <color rgb="FF000000"/>
-      <name val="Aptos Narrow"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="5">
@@ -213,55 +213,71 @@
   </borders>
   <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="44" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="4" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="3" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="3" fontId="8" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="44" fontId="6" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="44" fontId="8" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="2" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="2" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="3" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="3" fontId="7" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="3" fontId="7" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="4" fontId="7" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="169" fontId="9" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="169" fontId="1" fillId="3" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -281,6 +297,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -600,28 +620,26 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33EBFE00-5CAB-1A46-B0BC-D07B17BC850E}">
-  <dimension ref="A1:S10"/>
+  <dimension ref="A1:Q10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="22.33203125" customWidth="1"/>
-    <col min="3" max="3" width="13.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="16" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.5" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.1640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="21.6640625" customWidth="1"/>
-    <col min="10" max="10" width="17.1640625" customWidth="1"/>
-    <col min="12" max="12" width="18.1640625" customWidth="1"/>
+    <col min="3" max="3" width="14" style="7" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="16.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.1640625" customWidth="1"/>
+    <col min="9" max="16" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A1" s="6" t="s">
+    <row r="1" spans="1:17" s="12" customFormat="1" ht="51" x14ac:dyDescent="0.2">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="9" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="8" t="s">
@@ -630,198 +648,183 @@
       <c r="E1" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="F1" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="G1" s="8" t="s">
         <v>13</v>
       </c>
       <c r="H1" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="I1" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="K1" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="L1" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="M1" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="N1" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="I1" s="11" t="s">
+      <c r="O1" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="J1" s="11" t="s">
+      <c r="P1" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="K1" s="11" t="s">
+      <c r="Q1" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="L1" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="M1" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="N1" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="O1" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="P1" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="Q1" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="R1" s="6"/>
-      <c r="S1" s="5"/>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+    <row r="2" spans="1:17" s="23" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="B2" s="21" t="s">
+      <c r="B2" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="22">
+      <c r="C2" s="14">
         <v>374054.85547306883</v>
       </c>
-      <c r="D2" s="22">
+      <c r="D2" s="15">
         <v>11425477</v>
       </c>
-      <c r="E2" s="22">
+      <c r="E2" s="15">
         <v>28040181</v>
       </c>
-      <c r="F2" s="23">
-        <v>329792</v>
-      </c>
-      <c r="G2" s="23">
-        <v>82637</v>
-      </c>
-      <c r="H2" s="12"/>
-      <c r="I2" s="13"/>
-      <c r="J2" s="14">
+      <c r="F2" s="16">
+        <v>143828</v>
+      </c>
+      <c r="G2" s="16">
+        <v>35892</v>
+      </c>
+      <c r="H2" s="17">
+        <f>G2/D2*E2</f>
+        <v>88085.440673680409</v>
+      </c>
+      <c r="I2" s="18">
+        <f>G2/D2</f>
+        <v>3.1414005734727748E-3</v>
+      </c>
+      <c r="J2" s="18">
+        <f>F2/E2</f>
+        <v>5.1293534802788901E-3</v>
+      </c>
+      <c r="K2" s="18">
+        <f>(J2-I2)/I2</f>
+        <v>0.63282375498151155</v>
+      </c>
+      <c r="L2" s="19">
+        <f>F2-H2</f>
+        <v>55742.559326319591</v>
+      </c>
+      <c r="M2" s="20">
+        <f>C2/L2</f>
+        <v>6.7103997375386717</v>
+      </c>
+      <c r="N2" s="21"/>
+      <c r="O2" s="21"/>
+      <c r="P2" s="22">
         <v>0.99</v>
       </c>
-      <c r="K2" s="15"/>
-      <c r="L2" s="24">
-        <f>G2/D2*E2</f>
-        <v>202806.10055028775</v>
-      </c>
-      <c r="M2" s="16">
-        <f>G2/D2</f>
-        <v>7.2326958428081383E-3</v>
-      </c>
-      <c r="N2" s="16">
-        <f>F2/E2</f>
-        <v>1.1761407674222931E-2</v>
-      </c>
-      <c r="O2" s="17">
-        <f>(N2-M2)/M2</f>
-        <v>0.62614437684641977</v>
-      </c>
-      <c r="P2" s="18">
-        <f>F2-L2</f>
-        <v>126985.89944971225</v>
-      </c>
-      <c r="Q2" s="19">
-        <f>C2/P2</f>
-        <v>2.9456408711047364</v>
-      </c>
-      <c r="R2" s="4"/>
-      <c r="S2" s="7"/>
+      <c r="Q2" s="21"/>
     </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A3" s="21" t="s">
+    <row r="3" spans="1:17" s="23" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="B3" s="21" t="s">
+      <c r="B3" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="C3" s="22">
+      <c r="C3" s="14">
         <v>366145.38038958894</v>
       </c>
-      <c r="D3" s="22">
+      <c r="D3" s="15">
         <v>2522229</v>
       </c>
-      <c r="E3" s="22">
+      <c r="E3" s="15">
         <v>7763782</v>
       </c>
-      <c r="F3" s="23">
-        <v>98768</v>
-      </c>
-      <c r="G3" s="23">
-        <v>24271</v>
-      </c>
-      <c r="H3" s="12"/>
-      <c r="I3" s="12"/>
-      <c r="J3" s="14">
+      <c r="F3" s="16">
+        <v>47458</v>
+      </c>
+      <c r="G3" s="16">
+        <v>11632</v>
+      </c>
+      <c r="H3" s="17">
+        <f>G3/D3*E3</f>
+        <v>35804.961493980132</v>
+      </c>
+      <c r="I3" s="18">
+        <f>G3/D3</f>
+        <v>4.6117937744748795E-3</v>
+      </c>
+      <c r="J3" s="18">
+        <f>F3/E3</f>
+        <v>6.1127424752523965E-3</v>
+      </c>
+      <c r="K3" s="18">
+        <f>(J3-I3)/I3</f>
+        <v>0.32545876380788991</v>
+      </c>
+      <c r="L3" s="19">
+        <f>F3-H3</f>
+        <v>11653.038506019868</v>
+      </c>
+      <c r="M3" s="20">
+        <f>C3/L3</f>
+        <v>31.42059302390884</v>
+      </c>
+      <c r="N3" s="21"/>
+      <c r="O3" s="21"/>
+      <c r="P3" s="22">
         <v>0.99</v>
       </c>
-      <c r="K3" s="20"/>
-      <c r="L3" s="24">
-        <f>G3/D3*E3</f>
-        <v>74709.613172317026</v>
-      </c>
-      <c r="M3" s="16">
-        <f>G3/D3</f>
-        <v>9.6228375773968183E-3</v>
-      </c>
-      <c r="N3" s="16">
-        <f>F3/E3</f>
-        <v>1.2721634893921545E-2</v>
-      </c>
-      <c r="O3" s="17">
-        <f>(N3-M3)/M3</f>
-        <v>0.32202531650368116</v>
-      </c>
-      <c r="P3" s="18">
-        <f>F3-L3</f>
-        <v>24058.386827682974</v>
-      </c>
-      <c r="Q3" s="19">
-        <f>C3/P3</f>
-        <v>15.219032889116274</v>
-      </c>
-      <c r="R3" s="4"/>
-      <c r="S3" s="7"/>
+      <c r="Q3" s="24"/>
     </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A4" s="3"/>
       <c r="B4" s="3"/>
       <c r="E4" s="2"/>
       <c r="F4" s="3"/>
       <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
-      <c r="I4" s="1"/>
-      <c r="J4" s="3"/>
-      <c r="Q4" s="1"/>
+      <c r="M4" s="1"/>
     </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="E5" s="2"/>
       <c r="F5" s="3"/>
       <c r="G5" s="3"/>
-      <c r="H5" s="3"/>
-      <c r="I5" s="1"/>
-      <c r="J5" s="3"/>
-      <c r="N5" s="4"/>
-      <c r="Q5" s="1"/>
+      <c r="J5" s="4"/>
+      <c r="M5" s="1"/>
     </row>
-    <row r="6" spans="1:19" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:17" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="3"/>
       <c r="B6" s="3"/>
       <c r="E6" s="2"/>
       <c r="F6" s="3"/>
       <c r="G6" s="3"/>
-      <c r="H6" s="3"/>
-      <c r="I6" s="1"/>
-      <c r="J6" s="3"/>
-      <c r="N6" s="4"/>
-      <c r="Q6" s="1"/>
+      <c r="J6" s="4"/>
+      <c r="M6" s="1"/>
     </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="Q8" s="6"/>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="M8" s="5"/>
     </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="Q9" s="19"/>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="M9" s="6"/>
     </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="Q10" s="19"/>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="M10" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>